<commit_message>
Fix 20-sample test: SK indices were out of range (randint 2-5 vs valid 0-4)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_run/resultados_20_alumnos.xlsx
+++ b/test_run/resultados_20_alumnos.xlsx
@@ -1058,7 +1058,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generado: 05/05/2026 13:18</t>
+          <t>Generado: 05/05/2026 13:22</t>
         </is>
       </c>
     </row>
@@ -1145,7 +1145,7 @@
         <v>75</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>3.86</v>
+        <v>3.7</v>
       </c>
       <c r="I5" s="4" t="n">
         <v>100</v>
@@ -1178,16 +1178,16 @@
         </is>
       </c>
       <c r="E6" s="6" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F6" s="6" t="n">
         <v>20</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>4</v>
+        <v>3.3</v>
       </c>
       <c r="I6" s="6" t="n">
         <v>100</v>
@@ -1220,16 +1220,16 @@
         </is>
       </c>
       <c r="E7" s="4" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F7" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="G7" s="5" t="n">
-        <v>70</v>
+      <c r="G7" s="7" t="n">
+        <v>60</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>3.5</v>
+        <v>2.7</v>
       </c>
       <c r="I7" s="4" t="n">
         <v>100</v>
@@ -1262,16 +1262,16 @@
         </is>
       </c>
       <c r="E8" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F8" s="6" t="n">
         <v>20</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>3.29</v>
+        <v>2.9</v>
       </c>
       <c r="I8" s="6" t="n">
         <v>100</v>
@@ -1304,16 +1304,16 @@
         </is>
       </c>
       <c r="E9" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F9" s="4" t="n">
         <v>20</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>4</v>
+        <v>2.7</v>
       </c>
       <c r="I9" s="4" t="n">
         <v>100</v>
@@ -1346,16 +1346,16 @@
         </is>
       </c>
       <c r="E10" s="6" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="F10" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="G10" s="5" t="n">
-        <v>70</v>
+      <c r="G10" s="7" t="n">
+        <v>45</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>4.1</v>
+        <v>2.9</v>
       </c>
       <c r="I10" s="6" t="n">
         <v>100</v>
@@ -1388,16 +1388,16 @@
         </is>
       </c>
       <c r="E11" s="4" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F11" s="4" t="n">
         <v>20</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>4</v>
+        <v>2.8</v>
       </c>
       <c r="I11" s="4" t="n">
         <v>100</v>
@@ -1430,16 +1430,16 @@
         </is>
       </c>
       <c r="E12" s="6" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F12" s="6" t="n">
         <v>20</v>
       </c>
       <c r="G12" s="7" t="n">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="H12" s="6" t="n">
-        <v>4.12</v>
+        <v>2.7</v>
       </c>
       <c r="I12" s="6" t="n">
         <v>100</v>
@@ -1472,16 +1472,16 @@
         </is>
       </c>
       <c r="E13" s="4" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F13" s="4" t="n">
         <v>20</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>4.33</v>
+        <v>3.1</v>
       </c>
       <c r="I13" s="4" t="n">
         <v>100</v>
@@ -1514,16 +1514,16 @@
         </is>
       </c>
       <c r="E14" s="6" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="F14" s="6" t="n">
         <v>20</v>
       </c>
       <c r="G14" s="5" t="n">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="H14" s="6" t="n">
-        <v>3.8</v>
+        <v>2.2</v>
       </c>
       <c r="I14" s="6" t="n">
         <v>100</v>
@@ -1556,13 +1556,13 @@
         </is>
       </c>
       <c r="E15" s="4" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F15" s="4" t="n">
         <v>20</v>
       </c>
       <c r="G15" s="5" t="n">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="H15" s="4" t="n">
         <v>4</v>
@@ -1598,16 +1598,16 @@
         </is>
       </c>
       <c r="E16" s="6" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="F16" s="6" t="n">
         <v>20</v>
       </c>
       <c r="G16" s="5" t="n">
-        <v>95</v>
+        <v>70</v>
       </c>
       <c r="H16" s="6" t="n">
-        <v>3.88</v>
+        <v>3.6</v>
       </c>
       <c r="I16" s="6" t="n">
         <v>100</v>
@@ -1640,16 +1640,16 @@
         </is>
       </c>
       <c r="E17" s="4" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F17" s="4" t="n">
         <v>20</v>
       </c>
       <c r="G17" s="5" t="n">
-        <v>75</v>
+        <v>95</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>4</v>
+        <v>2.7</v>
       </c>
       <c r="I17" s="4" t="n">
         <v>100</v>
@@ -1682,16 +1682,16 @@
         </is>
       </c>
       <c r="E18" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F18" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="G18" s="7" t="n">
-        <v>60</v>
+      <c r="G18" s="5" t="n">
+        <v>70</v>
       </c>
       <c r="H18" s="6" t="n">
-        <v>4.33</v>
+        <v>2.7</v>
       </c>
       <c r="I18" s="6" t="n">
         <v>100</v>
@@ -1724,16 +1724,16 @@
         </is>
       </c>
       <c r="E19" s="4" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="F19" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="G19" s="5" t="n">
-        <v>75</v>
+      <c r="G19" s="7" t="n">
+        <v>60</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>4.22</v>
+        <v>3.1</v>
       </c>
       <c r="I19" s="4" t="n">
         <v>100</v>
@@ -1775,7 +1775,7 @@
         <v>75</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>3.8</v>
+        <v>3.6</v>
       </c>
       <c r="I20" s="6" t="n">
         <v>100</v>
@@ -1808,16 +1808,16 @@
         </is>
       </c>
       <c r="E21" s="4" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F21" s="4" t="n">
         <v>20</v>
       </c>
       <c r="G21" s="5" t="n">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>4</v>
+        <v>2.6</v>
       </c>
       <c r="I21" s="4" t="n">
         <v>100</v>
@@ -1850,16 +1850,16 @@
         </is>
       </c>
       <c r="E22" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F22" s="6" t="n">
         <v>20</v>
       </c>
       <c r="G22" s="5" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="H22" s="6" t="n">
-        <v>4.57</v>
+        <v>2.9</v>
       </c>
       <c r="I22" s="6" t="n">
         <v>100</v>
@@ -1901,7 +1901,7 @@
         <v>80</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>3.57</v>
+        <v>3.4</v>
       </c>
       <c r="I23" s="4" t="n">
         <v>100</v>
@@ -1934,16 +1934,16 @@
         </is>
       </c>
       <c r="E24" s="6" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="F24" s="6" t="n">
         <v>20</v>
       </c>
       <c r="G24" s="5" t="n">
-        <v>70</v>
+        <v>95</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>4.17</v>
+        <v>3.2</v>
       </c>
       <c r="I24" s="6" t="n">
         <v>100</v>
@@ -2458,9 +2458,9 @@
           <t>B</t>
         </is>
       </c>
-      <c r="G5" s="15" t="inlineStr">
-        <is>
-          <t>C</t>
+      <c r="G5" s="16" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="H5" s="15" t="inlineStr">
@@ -2473,39 +2473,39 @@
           <t>B</t>
         </is>
       </c>
-      <c r="J5" s="15" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="K5" s="16" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="L5" s="16" t="inlineStr">
-        <is>
-          <t>D</t>
+      <c r="J5" s="16" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="K5" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="L5" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="M5" s="16" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="N5" s="16" t="inlineStr">
         <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="O5" s="15" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="P5" s="15" t="inlineStr">
-        <is>
-          <t>D</t>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="O5" s="16" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="P5" s="16" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
       <c r="Q5" s="15" t="inlineStr">
@@ -2513,9 +2513,9 @@
           <t>A</t>
         </is>
       </c>
-      <c r="R5" s="16" t="inlineStr">
-        <is>
-          <t>D</t>
+      <c r="R5" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
       <c r="S5" s="15" t="inlineStr">
@@ -2523,9 +2523,9 @@
           <t>C</t>
         </is>
       </c>
-      <c r="T5" s="15" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="T5" s="16" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="U5" s="15" t="inlineStr">
@@ -2533,9 +2533,9 @@
           <t>D</t>
         </is>
       </c>
-      <c r="V5" s="16" t="inlineStr">
-        <is>
-          <t>D</t>
+      <c r="V5" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
       <c r="W5" s="15" t="inlineStr">
@@ -2568,9 +2568,9 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E6" s="15" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="E6" s="16" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
       <c r="F6" s="15" t="inlineStr">
@@ -2578,14 +2578,14 @@
           <t>B</t>
         </is>
       </c>
-      <c r="G6" s="15" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="H6" s="16" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="G6" s="16" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H6" s="15" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="I6" s="15" t="inlineStr">
@@ -2598,9 +2598,9 @@
           <t>A</t>
         </is>
       </c>
-      <c r="K6" s="15" t="inlineStr">
-        <is>
-          <t>B</t>
+      <c r="K6" s="16" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
       <c r="L6" s="15" t="inlineStr">
@@ -2608,29 +2608,29 @@
           <t>C</t>
         </is>
       </c>
-      <c r="M6" s="16" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="N6" s="16" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="O6" s="16" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="P6" s="15" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="Q6" s="15" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="M6" s="15" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="N6" s="15" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O6" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="P6" s="16" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="Q6" s="16" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="R6" s="16" t="inlineStr">
@@ -2643,14 +2643,14 @@
           <t>C</t>
         </is>
       </c>
-      <c r="T6" s="16" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="U6" s="15" t="inlineStr">
-        <is>
-          <t>D</t>
+      <c r="T6" s="15" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="U6" s="16" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="V6" s="15" t="inlineStr">
@@ -2658,9 +2658,9 @@
           <t>B</t>
         </is>
       </c>
-      <c r="W6" s="15" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="W6" s="16" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="X6" s="15" t="inlineStr">
@@ -2688,9 +2688,9 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E7" s="16" t="inlineStr">
-        <is>
-          <t>D</t>
+      <c r="E7" s="15" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
       <c r="F7" s="15" t="inlineStr">
@@ -2718,9 +2718,9 @@
           <t>A</t>
         </is>
       </c>
-      <c r="K7" s="16" t="inlineStr">
-        <is>
-          <t>C</t>
+      <c r="K7" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
       <c r="L7" s="15" t="inlineStr">
@@ -2728,19 +2728,19 @@
           <t>C</t>
         </is>
       </c>
-      <c r="M7" s="15" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="N7" s="16" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="O7" s="16" t="inlineStr">
-        <is>
-          <t>D</t>
+      <c r="M7" s="16" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="N7" s="15" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O7" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="P7" s="15" t="inlineStr">
@@ -2760,7 +2760,7 @@
       </c>
       <c r="S7" s="16" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="T7" s="15" t="inlineStr">
@@ -2773,14 +2773,14 @@
           <t>D</t>
         </is>
       </c>
-      <c r="V7" s="15" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="W7" s="15" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="V7" s="16" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="W7" s="16" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="X7" s="15" t="inlineStr">
@@ -2808,9 +2808,9 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E8" s="15" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="E8" s="16" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
       <c r="F8" s="15" t="inlineStr">
@@ -2820,7 +2820,7 @@
       </c>
       <c r="G8" s="16" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="H8" s="15" t="inlineStr">
@@ -2835,12 +2835,12 @@
       </c>
       <c r="J8" s="16" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="K8" s="16" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="L8" s="15" t="inlineStr">
@@ -2853,19 +2853,19 @@
           <t>D</t>
         </is>
       </c>
-      <c r="N8" s="16" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="O8" s="16" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="P8" s="16" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="N8" s="15" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O8" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="P8" s="15" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="Q8" s="15" t="inlineStr">
@@ -2873,14 +2873,14 @@
           <t>A</t>
         </is>
       </c>
-      <c r="R8" s="15" t="inlineStr">
-        <is>
-          <t>B</t>
+      <c r="R8" s="16" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="S8" s="16" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="T8" s="15" t="inlineStr">
@@ -2890,22 +2890,22 @@
       </c>
       <c r="U8" s="16" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="V8" s="16" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="W8" s="15" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="X8" s="16" t="inlineStr">
-        <is>
-          <t>A</t>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="W8" s="16" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="X8" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
     </row>
@@ -2930,7 +2930,7 @@
       </c>
       <c r="E9" s="16" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="F9" s="15" t="inlineStr">
@@ -2953,9 +2953,9 @@
           <t>D</t>
         </is>
       </c>
-      <c r="J9" s="16" t="inlineStr">
-        <is>
-          <t>B</t>
+      <c r="J9" s="15" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
       <c r="K9" s="15" t="inlineStr">
@@ -2963,14 +2963,14 @@
           <t>B</t>
         </is>
       </c>
-      <c r="L9" s="15" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="M9" s="15" t="inlineStr">
-        <is>
-          <t>D</t>
+      <c r="L9" s="16" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="M9" s="16" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="N9" s="15" t="inlineStr">
@@ -2978,14 +2978,14 @@
           <t>A</t>
         </is>
       </c>
-      <c r="O9" s="15" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="P9" s="15" t="inlineStr">
-        <is>
-          <t>D</t>
+      <c r="O9" s="16" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="P9" s="16" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
       <c r="Q9" s="15" t="inlineStr">
@@ -2998,9 +2998,9 @@
           <t>B</t>
         </is>
       </c>
-      <c r="S9" s="15" t="inlineStr">
-        <is>
-          <t>C</t>
+      <c r="S9" s="16" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
       <c r="T9" s="15" t="inlineStr">
@@ -3010,7 +3010,7 @@
       </c>
       <c r="U9" s="16" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="V9" s="15" t="inlineStr">
@@ -3023,9 +3023,9 @@
           <t>D</t>
         </is>
       </c>
-      <c r="X9" s="15" t="inlineStr">
-        <is>
-          <t>C</t>
+      <c r="X9" s="16" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -3048,9 +3048,9 @@
           <t>B</t>
         </is>
       </c>
-      <c r="E10" s="15" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="E10" s="16" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="F10" s="15" t="inlineStr">
@@ -3060,7 +3060,7 @@
       </c>
       <c r="G10" s="16" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="H10" s="15" t="inlineStr">
@@ -3068,9 +3068,9 @@
           <t>D</t>
         </is>
       </c>
-      <c r="I10" s="15" t="inlineStr">
-        <is>
-          <t>B</t>
+      <c r="I10" s="16" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
       <c r="J10" s="15" t="inlineStr">
@@ -3078,19 +3078,19 @@
           <t>A</t>
         </is>
       </c>
-      <c r="K10" s="15" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="L10" s="16" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="M10" s="16" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="K10" s="16" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="L10" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="M10" s="15" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="N10" s="16" t="inlineStr">
@@ -3098,14 +3098,14 @@
           <t>D</t>
         </is>
       </c>
-      <c r="O10" s="16" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="P10" s="15" t="inlineStr">
-        <is>
-          <t>D</t>
+      <c r="O10" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="P10" s="16" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
       <c r="Q10" s="15" t="inlineStr">
@@ -3113,19 +3113,19 @@
           <t>A</t>
         </is>
       </c>
-      <c r="R10" s="16" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="S10" s="15" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="T10" s="16" t="inlineStr">
-        <is>
-          <t>D</t>
+      <c r="R10" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="S10" s="16" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="T10" s="15" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
       <c r="U10" s="15" t="inlineStr">
@@ -3143,9 +3143,9 @@
           <t>A</t>
         </is>
       </c>
-      <c r="X10" s="15" t="inlineStr">
-        <is>
-          <t>C</t>
+      <c r="X10" s="16" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
     </row>
@@ -3168,34 +3168,34 @@
           <t>B</t>
         </is>
       </c>
-      <c r="E11" s="16" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="F11" s="16" t="inlineStr">
-        <is>
-          <t>C</t>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F11" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
       <c r="G11" s="16" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H11" s="16" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="I11" s="15" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="J11" s="16" t="inlineStr">
-        <is>
-          <t>C</t>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I11" s="16" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="J11" s="15" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
       <c r="K11" s="16" t="inlineStr">
@@ -3203,19 +3203,19 @@
           <t>C</t>
         </is>
       </c>
-      <c r="L11" s="15" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="M11" s="16" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="N11" s="15" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="L11" s="16" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M11" s="15" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="N11" s="16" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
       <c r="O11" s="16" t="inlineStr">
@@ -3223,29 +3223,29 @@
           <t>A</t>
         </is>
       </c>
-      <c r="P11" s="15" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="Q11" s="16" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="R11" s="15" t="inlineStr">
-        <is>
-          <t>B</t>
+      <c r="P11" s="16" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="Q11" s="15" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="R11" s="16" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="S11" s="16" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="T11" s="15" t="inlineStr">
-        <is>
-          <t>A</t>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="T11" s="16" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="U11" s="15" t="inlineStr">
@@ -3255,12 +3255,12 @@
       </c>
       <c r="V11" s="16" t="inlineStr">
         <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="W11" s="15" t="inlineStr">
-        <is>
-          <t>A</t>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="W11" s="16" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="X11" s="15" t="inlineStr">
@@ -3288,9 +3288,9 @@
           <t>B</t>
         </is>
       </c>
-      <c r="E12" s="15" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="E12" s="16" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="F12" s="16" t="inlineStr">
@@ -3298,19 +3298,19 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G12" s="16" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="H12" s="16" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="I12" s="15" t="inlineStr">
-        <is>
-          <t>B</t>
+      <c r="G12" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H12" s="15" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="I12" s="16" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="J12" s="15" t="inlineStr">
@@ -3323,29 +3323,29 @@
           <t>C</t>
         </is>
       </c>
-      <c r="L12" s="16" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="M12" s="16" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="N12" s="16" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="O12" s="15" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="P12" s="15" t="inlineStr">
-        <is>
-          <t>D</t>
+      <c r="L12" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="M12" s="15" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="N12" s="15" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O12" s="16" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="P12" s="16" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="Q12" s="15" t="inlineStr">
@@ -3353,9 +3353,9 @@
           <t>A</t>
         </is>
       </c>
-      <c r="R12" s="15" t="inlineStr">
-        <is>
-          <t>B</t>
+      <c r="R12" s="16" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
       <c r="S12" s="15" t="inlineStr">
@@ -3363,29 +3363,29 @@
           <t>C</t>
         </is>
       </c>
-      <c r="T12" s="15" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="U12" s="16" t="inlineStr">
-        <is>
-          <t>C</t>
+      <c r="T12" s="16" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="U12" s="15" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="V12" s="16" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="W12" s="16" t="inlineStr">
         <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="X12" s="15" t="inlineStr">
-        <is>
-          <t>C</t>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X12" s="16" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -3408,9 +3408,9 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E13" s="16" t="inlineStr">
-        <is>
-          <t>B</t>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
       <c r="F13" s="15" t="inlineStr">
@@ -3423,9 +3423,9 @@
           <t>C</t>
         </is>
       </c>
-      <c r="H13" s="15" t="inlineStr">
-        <is>
-          <t>D</t>
+      <c r="H13" s="16" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
       <c r="I13" s="15" t="inlineStr">
@@ -3443,9 +3443,9 @@
           <t>B</t>
         </is>
       </c>
-      <c r="L13" s="16" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="L13" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="M13" s="15" t="inlineStr">
@@ -3453,9 +3453,9 @@
           <t>D</t>
         </is>
       </c>
-      <c r="N13" s="16" t="inlineStr">
-        <is>
-          <t>D</t>
+      <c r="N13" s="15" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
       <c r="O13" s="15" t="inlineStr">
@@ -3490,12 +3490,12 @@
       </c>
       <c r="U13" s="16" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="V13" s="16" t="inlineStr">
-        <is>
-          <t>A</t>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="V13" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
       <c r="W13" s="15" t="inlineStr">
@@ -3503,9 +3503,9 @@
           <t>A</t>
         </is>
       </c>
-      <c r="X13" s="16" t="inlineStr">
-        <is>
-          <t>D</t>
+      <c r="X13" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
     </row>
@@ -3533,14 +3533,14 @@
           <t>A</t>
         </is>
       </c>
-      <c r="F14" s="15" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="G14" s="16" t="inlineStr">
-        <is>
-          <t>D</t>
+      <c r="F14" s="16" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="G14" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="H14" s="15" t="inlineStr">
@@ -3558,9 +3558,9 @@
           <t>A</t>
         </is>
       </c>
-      <c r="K14" s="16" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="K14" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
       <c r="L14" s="15" t="inlineStr">
@@ -3568,14 +3568,14 @@
           <t>C</t>
         </is>
       </c>
-      <c r="M14" s="15" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="N14" s="15" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="M14" s="16" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="N14" s="16" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
       <c r="O14" s="15" t="inlineStr">
@@ -3583,9 +3583,9 @@
           <t>C</t>
         </is>
       </c>
-      <c r="P14" s="15" t="inlineStr">
-        <is>
-          <t>D</t>
+      <c r="P14" s="16" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="Q14" s="15" t="inlineStr">
@@ -3593,14 +3593,14 @@
           <t>A</t>
         </is>
       </c>
-      <c r="R14" s="16" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="S14" s="15" t="inlineStr">
-        <is>
-          <t>C</t>
+      <c r="R14" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="S14" s="16" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
       <c r="T14" s="15" t="inlineStr">
@@ -3608,9 +3608,9 @@
           <t>A</t>
         </is>
       </c>
-      <c r="U14" s="15" t="inlineStr">
-        <is>
-          <t>D</t>
+      <c r="U14" s="16" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="V14" s="15" t="inlineStr">
@@ -3618,14 +3618,14 @@
           <t>B</t>
         </is>
       </c>
-      <c r="W14" s="16" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="X14" s="16" t="inlineStr">
-        <is>
-          <t>D</t>
+      <c r="W14" s="15" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="X14" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
     </row>
@@ -3663,9 +3663,9 @@
           <t>C</t>
         </is>
       </c>
-      <c r="H15" s="15" t="inlineStr">
-        <is>
-          <t>D</t>
+      <c r="H15" s="16" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
       <c r="I15" s="15" t="inlineStr">
@@ -3698,9 +3698,9 @@
           <t>A</t>
         </is>
       </c>
-      <c r="O15" s="15" t="inlineStr">
-        <is>
-          <t>C</t>
+      <c r="O15" s="16" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
       <c r="P15" s="15" t="inlineStr">
@@ -3723,29 +3723,29 @@
           <t>C</t>
         </is>
       </c>
-      <c r="T15" s="15" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="U15" s="15" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="V15" s="15" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="W15" s="15" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="X15" s="16" t="inlineStr">
-        <is>
-          <t>B</t>
+      <c r="T15" s="16" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="U15" s="16" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="V15" s="16" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="W15" s="16" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X15" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
     </row>
@@ -3808,9 +3808,9 @@
           <t>C</t>
         </is>
       </c>
-      <c r="M16" s="16" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="M16" s="15" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="N16" s="15" t="inlineStr">
@@ -3818,9 +3818,9 @@
           <t>A</t>
         </is>
       </c>
-      <c r="O16" s="16" t="inlineStr">
-        <is>
-          <t>D</t>
+      <c r="O16" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="P16" s="15" t="inlineStr">
@@ -3828,9 +3828,9 @@
           <t>D</t>
         </is>
       </c>
-      <c r="Q16" s="16" t="inlineStr">
-        <is>
-          <t>C</t>
+      <c r="Q16" s="15" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
       <c r="R16" s="15" t="inlineStr">
@@ -3853,19 +3853,19 @@
           <t>D</t>
         </is>
       </c>
-      <c r="V16" s="16" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="W16" s="16" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="X16" s="15" t="inlineStr">
-        <is>
-          <t>C</t>
+      <c r="V16" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="W16" s="15" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="X16" s="16" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -3888,24 +3888,24 @@
           <t>B</t>
         </is>
       </c>
-      <c r="E17" s="15" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="F17" s="16" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="G17" s="16" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="H17" s="16" t="inlineStr">
-        <is>
-          <t>B</t>
+      <c r="E17" s="16" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="F17" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G17" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H17" s="15" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="I17" s="15" t="inlineStr">
@@ -3928,34 +3928,34 @@
           <t>C</t>
         </is>
       </c>
-      <c r="M17" s="16" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="N17" s="15" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="O17" s="16" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="P17" s="15" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="Q17" s="16" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="R17" s="15" t="inlineStr">
-        <is>
-          <t>B</t>
+      <c r="M17" s="15" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="N17" s="16" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="O17" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="P17" s="16" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Q17" s="15" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="R17" s="16" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="S17" s="15" t="inlineStr">
@@ -3963,9 +3963,9 @@
           <t>C</t>
         </is>
       </c>
-      <c r="T17" s="16" t="inlineStr">
-        <is>
-          <t>D</t>
+      <c r="T17" s="15" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
       <c r="U17" s="15" t="inlineStr">
@@ -3978,9 +3978,9 @@
           <t>B</t>
         </is>
       </c>
-      <c r="W17" s="15" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="W17" s="16" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="X17" s="16" t="inlineStr">
@@ -4008,9 +4008,9 @@
           <t>B</t>
         </is>
       </c>
-      <c r="E18" s="15" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="E18" s="16" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="F18" s="15" t="inlineStr">
@@ -4018,9 +4018,9 @@
           <t>B</t>
         </is>
       </c>
-      <c r="G18" s="15" t="inlineStr">
-        <is>
-          <t>C</t>
+      <c r="G18" s="16" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="H18" s="16" t="inlineStr">
@@ -4030,7 +4030,7 @@
       </c>
       <c r="I18" s="16" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J18" s="15" t="inlineStr">
@@ -4053,9 +4053,9 @@
           <t>D</t>
         </is>
       </c>
-      <c r="N18" s="15" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="N18" s="16" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="O18" s="15" t="inlineStr">
@@ -4063,24 +4063,24 @@
           <t>C</t>
         </is>
       </c>
-      <c r="P18" s="15" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="Q18" s="16" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="R18" s="15" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="S18" s="16" t="inlineStr">
-        <is>
-          <t>B</t>
+      <c r="P18" s="16" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Q18" s="15" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="R18" s="16" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="S18" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="T18" s="15" t="inlineStr">
@@ -4088,14 +4088,14 @@
           <t>A</t>
         </is>
       </c>
-      <c r="U18" s="15" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="V18" s="16" t="inlineStr">
-        <is>
-          <t>C</t>
+      <c r="U18" s="16" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="V18" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
       <c r="W18" s="15" t="inlineStr">
@@ -4150,12 +4150,12 @@
       </c>
       <c r="I19" s="16" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J19" s="16" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="K19" s="15" t="inlineStr">
@@ -4183,19 +4183,19 @@
           <t>C</t>
         </is>
       </c>
-      <c r="P19" s="16" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="Q19" s="16" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="R19" s="15" t="inlineStr">
-        <is>
-          <t>B</t>
+      <c r="P19" s="15" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="Q19" s="15" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="R19" s="16" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="S19" s="15" t="inlineStr">
@@ -4203,9 +4203,9 @@
           <t>C</t>
         </is>
       </c>
-      <c r="T19" s="15" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="T19" s="16" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="U19" s="15" t="inlineStr">
@@ -4218,14 +4218,14 @@
           <t>B</t>
         </is>
       </c>
-      <c r="W19" s="15" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="X19" s="16" t="inlineStr">
-        <is>
-          <t>B</t>
+      <c r="W19" s="16" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="X19" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
     </row>
@@ -4248,9 +4248,9 @@
           <t>B</t>
         </is>
       </c>
-      <c r="E20" s="16" t="inlineStr">
-        <is>
-          <t>B</t>
+      <c r="E20" s="15" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
       <c r="F20" s="15" t="inlineStr">
@@ -4273,9 +4273,9 @@
           <t>B</t>
         </is>
       </c>
-      <c r="J20" s="15" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="J20" s="16" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="K20" s="15" t="inlineStr">
@@ -4283,14 +4283,14 @@
           <t>B</t>
         </is>
       </c>
-      <c r="L20" s="15" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="M20" s="15" t="inlineStr">
-        <is>
-          <t>D</t>
+      <c r="L20" s="16" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M20" s="16" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
       <c r="N20" s="15" t="inlineStr">
@@ -4313,19 +4313,19 @@
           <t>A</t>
         </is>
       </c>
-      <c r="R20" s="16" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="S20" s="15" t="inlineStr">
-        <is>
-          <t>C</t>
+      <c r="R20" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="S20" s="16" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
       <c r="T20" s="16" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="U20" s="15" t="inlineStr">
@@ -4333,9 +4333,9 @@
           <t>D</t>
         </is>
       </c>
-      <c r="V20" s="16" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="V20" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
       <c r="W20" s="15" t="inlineStr">
@@ -4368,19 +4368,19 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E21" s="15" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="F21" s="15" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="G21" s="16" t="inlineStr">
-        <is>
-          <t>D</t>
+      <c r="E21" s="16" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="F21" s="16" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G21" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="H21" s="15" t="inlineStr">
@@ -4400,7 +4400,7 @@
       </c>
       <c r="K21" s="16" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="L21" s="15" t="inlineStr">
@@ -4418,9 +4418,9 @@
           <t>A</t>
         </is>
       </c>
-      <c r="O21" s="16" t="inlineStr">
-        <is>
-          <t>D</t>
+      <c r="O21" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="P21" s="15" t="inlineStr">
@@ -4443,14 +4443,14 @@
           <t>C</t>
         </is>
       </c>
-      <c r="T21" s="16" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="U21" s="16" t="inlineStr">
-        <is>
-          <t>B</t>
+      <c r="T21" s="15" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="U21" s="15" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="V21" s="15" t="inlineStr">
@@ -4463,9 +4463,9 @@
           <t>A</t>
         </is>
       </c>
-      <c r="X21" s="15" t="inlineStr">
-        <is>
-          <t>C</t>
+      <c r="X21" s="16" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -4498,14 +4498,14 @@
           <t>B</t>
         </is>
       </c>
-      <c r="G22" s="15" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="H22" s="16" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="G22" s="16" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H22" s="15" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="I22" s="15" t="inlineStr">
@@ -4543,9 +4543,9 @@
           <t>C</t>
         </is>
       </c>
-      <c r="P22" s="15" t="inlineStr">
-        <is>
-          <t>D</t>
+      <c r="P22" s="16" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="Q22" s="15" t="inlineStr">
@@ -4558,14 +4558,14 @@
           <t>B</t>
         </is>
       </c>
-      <c r="S22" s="16" t="inlineStr">
-        <is>
-          <t>B</t>
+      <c r="S22" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="T22" s="16" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="U22" s="15" t="inlineStr">
@@ -4573,9 +4573,9 @@
           <t>D</t>
         </is>
       </c>
-      <c r="V22" s="16" t="inlineStr">
-        <is>
-          <t>D</t>
+      <c r="V22" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
       <c r="W22" s="15" t="inlineStr">
@@ -4583,9 +4583,9 @@
           <t>A</t>
         </is>
       </c>
-      <c r="X22" s="15" t="inlineStr">
-        <is>
-          <t>C</t>
+      <c r="X22" s="16" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
     </row>
@@ -4608,9 +4608,9 @@
           <t>B</t>
         </is>
       </c>
-      <c r="E23" s="16" t="inlineStr">
-        <is>
-          <t>B</t>
+      <c r="E23" s="15" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
       <c r="F23" s="15" t="inlineStr">
@@ -4653,14 +4653,14 @@
           <t>D</t>
         </is>
       </c>
-      <c r="N23" s="16" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="O23" s="16" t="inlineStr">
-        <is>
-          <t>D</t>
+      <c r="N23" s="15" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O23" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="P23" s="15" t="inlineStr">
@@ -4680,17 +4680,17 @@
       </c>
       <c r="S23" s="16" t="inlineStr">
         <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="T23" s="16" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="U23" s="16" t="inlineStr">
-        <is>
-          <t>B</t>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="T23" s="15" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="U23" s="15" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="V23" s="15" t="inlineStr">
@@ -4716,7 +4716,7 @@
         </is>
       </c>
       <c r="E25" s="18" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="F25" s="15" t="n">
         <v>85</v>
@@ -4724,56 +4724,56 @@
       <c r="G25" s="18" t="n">
         <v>60</v>
       </c>
-      <c r="H25" s="18" t="n">
-        <v>70</v>
+      <c r="H25" s="15" t="n">
+        <v>80</v>
       </c>
       <c r="I25" s="18" t="n">
-        <v>75</v>
+        <v>60</v>
       </c>
       <c r="J25" s="15" t="n">
         <v>80</v>
       </c>
       <c r="K25" s="18" t="n">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="L25" s="15" t="n">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="M25" s="18" t="n">
+        <v>75</v>
+      </c>
+      <c r="N25" s="18" t="n">
+        <v>70</v>
+      </c>
+      <c r="O25" s="18" t="n">
+        <v>75</v>
+      </c>
+      <c r="P25" s="18" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q25" s="15" t="n">
+        <v>90</v>
+      </c>
+      <c r="R25" s="18" t="n">
         <v>65</v>
       </c>
-      <c r="N25" s="18" t="n">
-        <v>60</v>
-      </c>
-      <c r="O25" s="18" t="n">
+      <c r="S25" s="18" t="n">
         <v>55</v>
-      </c>
-      <c r="P25" s="15" t="n">
-        <v>90</v>
-      </c>
-      <c r="Q25" s="18" t="n">
-        <v>70</v>
-      </c>
-      <c r="R25" s="18" t="n">
-        <v>75</v>
-      </c>
-      <c r="S25" s="18" t="n">
-        <v>65</v>
       </c>
       <c r="T25" s="18" t="n">
         <v>60</v>
       </c>
       <c r="U25" s="18" t="n">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="V25" s="18" t="n">
+        <v>75</v>
+      </c>
+      <c r="W25" s="18" t="n">
         <v>55</v>
       </c>
-      <c r="W25" s="15" t="n">
-        <v>80</v>
-      </c>
       <c r="X25" s="18" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>
@@ -4916,17 +4916,13 @@
         </is>
       </c>
       <c r="E3" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="F3" s="20" t="n">
         <v>5</v>
       </c>
-      <c r="F3" s="20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G3" s="20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="G3" s="20" t="n">
+        <v>4</v>
       </c>
       <c r="H3" s="20" t="n">
         <v>5</v>
@@ -4935,24 +4931,22 @@
         <v>4</v>
       </c>
       <c r="J3" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="K3" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="L3" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="M3" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="N3" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="K3" s="20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L3" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="M3" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="N3" s="20" t="n">
-        <v>3</v>
-      </c>
       <c r="O3" s="21" t="n">
-        <v>3.86</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="4">
@@ -4977,39 +4971,37 @@
         </is>
       </c>
       <c r="E4" s="22" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F4" s="22" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G4" s="22" t="n">
         <v>5</v>
       </c>
       <c r="H4" s="22" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I4" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="J4" s="22" t="n">
         <v>3</v>
       </c>
-      <c r="J4" s="22" t="n">
+      <c r="K4" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="L4" s="22" t="n">
         <v>5</v>
       </c>
-      <c r="K4" s="22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L4" s="22" t="n">
-        <v>3</v>
-      </c>
       <c r="M4" s="22" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N4" s="22" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O4" s="21" t="n">
-        <v>4</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="5">
@@ -5034,37 +5026,37 @@
         </is>
       </c>
       <c r="E5" s="20" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F5" s="20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G5" s="20" t="n">
         <v>3</v>
       </c>
       <c r="H5" s="20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I5" s="20" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J5" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K5" s="20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L5" s="20" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M5" s="20" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="N5" s="20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O5" s="21" t="n">
-        <v>3.5</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="6">
@@ -5089,43 +5081,37 @@
         </is>
       </c>
       <c r="E6" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="F6" s="22" t="n">
         <v>3</v>
       </c>
-      <c r="F6" s="22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="G6" s="22" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H6" s="22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I6" s="22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J6" s="22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K6" s="22" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L6" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="M6" s="22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N6" s="22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="M6" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="N6" s="22" t="n">
+        <v>4</v>
       </c>
       <c r="O6" s="21" t="n">
-        <v>3.29</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="7">
@@ -5149,42 +5135,38 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E7" s="20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="E7" s="20" t="n">
+        <v>3</v>
       </c>
       <c r="F7" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="G7" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="I7" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="J7" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="K7" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="G7" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="H7" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="I7" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="J7" s="20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K7" s="20" t="n">
-        <v>5</v>
-      </c>
       <c r="L7" s="20" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M7" s="20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N7" s="20" t="n">
         <v>5</v>
       </c>
       <c r="O7" s="21" t="n">
-        <v>4</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="8">
@@ -5209,10 +5191,10 @@
         </is>
       </c>
       <c r="E8" s="22" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F8" s="22" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G8" s="22" t="n">
         <v>5</v>
@@ -5221,25 +5203,25 @@
         <v>3</v>
       </c>
       <c r="I8" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="J8" s="22" t="n">
         <v>3</v>
       </c>
-      <c r="J8" s="22" t="n">
-        <v>4</v>
-      </c>
       <c r="K8" s="22" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="L8" s="22" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="M8" s="22" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N8" s="22" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O8" s="21" t="n">
-        <v>4.1</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="9">
@@ -5267,36 +5249,34 @@
         <v>3</v>
       </c>
       <c r="F9" s="20" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G9" s="20" t="n">
         <v>4</v>
       </c>
       <c r="H9" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="I9" s="20" t="n">
         <v>4</v>
-      </c>
-      <c r="I9" s="20" t="n">
-        <v>3</v>
       </c>
       <c r="J9" s="20" t="n">
         <v>5</v>
       </c>
-      <c r="K9" s="20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="K9" s="20" t="n">
+        <v>1</v>
       </c>
       <c r="L9" s="20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M9" s="20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N9" s="20" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O9" s="21" t="n">
-        <v>4</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="10">
@@ -5321,41 +5301,37 @@
         </is>
       </c>
       <c r="E10" s="22" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F10" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="G10" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="H10" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="I10" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="J10" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="L10" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="G10" s="22" t="n">
-        <v>5</v>
-      </c>
-      <c r="H10" s="22" t="n">
+      <c r="M10" s="22" t="n">
         <v>3</v>
-      </c>
-      <c r="I10" s="22" t="n">
-        <v>3</v>
-      </c>
-      <c r="J10" s="22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K10" s="22" t="n">
-        <v>5</v>
-      </c>
-      <c r="L10" s="22" t="n">
-        <v>5</v>
-      </c>
-      <c r="M10" s="22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
       </c>
       <c r="N10" s="22" t="n">
         <v>3</v>
       </c>
       <c r="O10" s="21" t="n">
-        <v>4.12</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="11">
@@ -5383,42 +5359,34 @@
         <v>3</v>
       </c>
       <c r="F11" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="G11" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="I11" s="20" t="n">
         <v>5</v>
       </c>
-      <c r="G11" s="20" t="n">
+      <c r="J11" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="K11" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="L11" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="M11" s="20" t="n">
         <v>5</v>
       </c>
-      <c r="H11" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="I11" s="20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J11" s="20" t="n">
-        <v>5</v>
-      </c>
-      <c r="K11" s="20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L11" s="20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M11" s="20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="N11" s="20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O11" s="21" t="n">
-        <v>4.33</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="12">
@@ -5442,48 +5410,38 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E12" s="22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="E12" s="22" t="n">
+        <v>5</v>
       </c>
       <c r="F12" s="22" t="n">
         <v>3</v>
       </c>
       <c r="G12" s="22" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H12" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="I12" s="22" t="n">
         <v>3</v>
       </c>
-      <c r="I12" s="22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="J12" s="22" t="n">
-        <v>4</v>
-      </c>
-      <c r="K12" s="22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>2</v>
+      </c>
+      <c r="K12" s="22" t="n">
+        <v>2</v>
       </c>
       <c r="L12" s="22" t="n">
-        <v>5</v>
-      </c>
-      <c r="M12" s="22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N12" s="22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>2</v>
+      </c>
+      <c r="M12" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="N12" s="22" t="n">
+        <v>1</v>
       </c>
       <c r="O12" s="21" t="n">
-        <v>3.8</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="13">
@@ -5508,44 +5466,34 @@
         </is>
       </c>
       <c r="E13" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="F13" s="20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G13" s="20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>4</v>
+      </c>
+      <c r="F13" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="G13" s="20" t="n">
+        <v>5</v>
       </c>
       <c r="H13" s="20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I13" s="20" t="n">
         <v>5</v>
       </c>
       <c r="J13" s="20" t="n">
-        <v>5</v>
-      </c>
-      <c r="K13" s="20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L13" s="20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>4</v>
+      </c>
+      <c r="K13" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="L13" s="20" t="n">
+        <v>4</v>
       </c>
       <c r="M13" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="N13" s="20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="N13" s="20" t="n">
+        <v>3</v>
       </c>
       <c r="O13" s="21" t="n">
         <v>4</v>
@@ -5573,41 +5521,37 @@
         </is>
       </c>
       <c r="E14" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="G14" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="H14" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="I14" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="J14" s="22" t="n">
         <v>5</v>
       </c>
-      <c r="F14" s="22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G14" s="22" t="n">
+      <c r="K14" s="22" t="n">
         <v>5</v>
-      </c>
-      <c r="H14" s="22" t="n">
-        <v>3</v>
-      </c>
-      <c r="I14" s="22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J14" s="22" t="n">
-        <v>3</v>
-      </c>
-      <c r="K14" s="22" t="n">
-        <v>3</v>
       </c>
       <c r="L14" s="22" t="n">
         <v>5</v>
       </c>
       <c r="M14" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="N14" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="N14" s="22" t="n">
-        <v>3</v>
-      </c>
       <c r="O14" s="21" t="n">
-        <v>3.88</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="15">
@@ -5632,39 +5576,37 @@
         </is>
       </c>
       <c r="E15" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="F15" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="F15" s="20" t="n">
+      <c r="G15" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="G15" s="20" t="n">
+      <c r="H15" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="I15" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="J15" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="K15" s="20" t="n">
         <v>5</v>
       </c>
-      <c r="H15" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="I15" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="J15" s="20" t="n">
-        <v>5</v>
-      </c>
-      <c r="K15" s="20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="L15" s="20" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M15" s="20" t="n">
         <v>3</v>
       </c>
       <c r="N15" s="20" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="O15" s="21" t="n">
-        <v>4</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="16">
@@ -5688,40 +5630,38 @@
           <t>B</t>
         </is>
       </c>
-      <c r="E16" s="22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="E16" s="22" t="n">
+        <v>1</v>
       </c>
       <c r="F16" s="22" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G16" s="22" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H16" s="22" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I16" s="22" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J16" s="22" t="n">
         <v>5</v>
       </c>
       <c r="K16" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="L16" s="22" t="n">
         <v>5</v>
       </c>
-      <c r="L16" s="22" t="n">
-        <v>3</v>
-      </c>
       <c r="M16" s="22" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N16" s="22" t="n">
         <v>3</v>
       </c>
       <c r="O16" s="21" t="n">
-        <v>4.33</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="17">
@@ -5746,39 +5686,37 @@
         </is>
       </c>
       <c r="E17" s="20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F17" s="20" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G17" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="H17" s="20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="H17" s="20" t="n">
+        <v>2</v>
       </c>
       <c r="I17" s="20" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J17" s="20" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K17" s="20" t="n">
         <v>3</v>
       </c>
       <c r="L17" s="20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M17" s="20" t="n">
         <v>5</v>
       </c>
       <c r="N17" s="20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O17" s="21" t="n">
-        <v>4.22</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="18">
@@ -5803,47 +5741,37 @@
         </is>
       </c>
       <c r="E18" s="22" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F18" s="22" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G18" s="22" t="n">
-        <v>3</v>
-      </c>
-      <c r="H18" s="22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>2</v>
+      </c>
+      <c r="H18" s="22" t="n">
+        <v>2</v>
       </c>
       <c r="I18" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="J18" s="22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K18" s="22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L18" s="22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="J18" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="K18" s="22" t="n">
+        <v>5</v>
+      </c>
+      <c r="L18" s="22" t="n">
+        <v>5</v>
       </c>
       <c r="M18" s="22" t="n">
         <v>5</v>
       </c>
-      <c r="N18" s="22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="N18" s="22" t="n">
+        <v>3</v>
       </c>
       <c r="O18" s="21" t="n">
-        <v>3.8</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="19">
@@ -5868,39 +5796,37 @@
         </is>
       </c>
       <c r="E19" s="20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F19" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="G19" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="H19" s="20" t="n">
         <v>5</v>
-      </c>
-      <c r="G19" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="H19" s="20" t="n">
-        <v>3</v>
       </c>
       <c r="I19" s="20" t="n">
         <v>3</v>
       </c>
       <c r="J19" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="K19" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="L19" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="M19" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="N19" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="K19" s="20" t="n">
-        <v>5</v>
-      </c>
-      <c r="L19" s="20" t="n">
-        <v>5</v>
-      </c>
-      <c r="M19" s="20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N19" s="20" t="n">
-        <v>3</v>
-      </c>
       <c r="O19" s="21" t="n">
-        <v>4</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="20">
@@ -5925,43 +5851,37 @@
         </is>
       </c>
       <c r="E20" s="22" t="n">
-        <v>5</v>
-      </c>
-      <c r="F20" s="22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>2</v>
+      </c>
+      <c r="F20" s="22" t="n">
+        <v>3</v>
       </c>
       <c r="G20" s="22" t="n">
         <v>5</v>
       </c>
       <c r="H20" s="22" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I20" s="22" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J20" s="22" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K20" s="22" t="n">
         <v>5</v>
       </c>
-      <c r="L20" s="22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M20" s="22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="L20" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="M20" s="22" t="n">
+        <v>2</v>
       </c>
       <c r="N20" s="22" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O20" s="21" t="n">
-        <v>4.57</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="21">
@@ -5986,18 +5906,16 @@
         </is>
       </c>
       <c r="E21" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="G21" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="H21" s="20" t="n">
         <v>5</v>
-      </c>
-      <c r="F21" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="G21" s="20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H21" s="20" t="n">
-        <v>3</v>
       </c>
       <c r="I21" s="20" t="n">
         <v>4</v>
@@ -6005,24 +5923,20 @@
       <c r="J21" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="K21" s="20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="K21" s="20" t="n">
+        <v>2</v>
       </c>
       <c r="L21" s="20" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M21" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="N21" s="20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="N21" s="20" t="n">
+        <v>4</v>
       </c>
       <c r="O21" s="21" t="n">
-        <v>3.57</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="22">
@@ -6046,46 +5960,38 @@
           <t>B</t>
         </is>
       </c>
-      <c r="E22" s="22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F22" s="22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="E22" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="F22" s="22" t="n">
+        <v>4</v>
       </c>
       <c r="G22" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="H22" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="I22" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="J22" s="22" t="n">
         <v>5</v>
       </c>
-      <c r="H22" s="22" t="n">
+      <c r="K22" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="L22" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="M22" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="I22" s="22" t="n">
+      <c r="N22" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="J22" s="22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K22" s="22" t="n">
-        <v>4</v>
-      </c>
-      <c r="L22" s="22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M22" s="22" t="n">
-        <v>3</v>
-      </c>
-      <c r="N22" s="22" t="n">
-        <v>5</v>
-      </c>
       <c r="O22" s="21" t="n">
-        <v>4.17</v>
+        <v>3.2</v>
       </c>
     </row>
   </sheetData>
@@ -6145,7 +6051,7 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6">
@@ -6155,7 +6061,7 @@
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
@@ -6175,7 +6081,7 @@
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9">
@@ -6185,7 +6091,7 @@
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10">
@@ -6195,7 +6101,7 @@
         </is>
       </c>
       <c r="B10" s="6" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11">
@@ -6205,7 +6111,7 @@
         </is>
       </c>
       <c r="B11" s="4" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="12">
@@ -6215,7 +6121,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13">
@@ -6225,7 +6131,7 @@
         </is>
       </c>
       <c r="B13" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14">
@@ -6235,7 +6141,7 @@
         </is>
       </c>
       <c r="B14" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15">
@@ -6245,7 +6151,7 @@
         </is>
       </c>
       <c r="B15" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -6284,7 +6190,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generado: 05/05/2026 13:18</t>
+          <t>Generado: 05/05/2026 13:22</t>
         </is>
       </c>
     </row>
@@ -6345,7 +6251,7 @@
         <v>75</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>3.86</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="6">
@@ -6370,10 +6276,10 @@
         </is>
       </c>
       <c r="E6" s="6" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>4</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="7">
@@ -6398,10 +6304,10 @@
         </is>
       </c>
       <c r="E7" s="4" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>3.5</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="8">
@@ -6426,10 +6332,10 @@
         </is>
       </c>
       <c r="E8" s="6" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>3.29</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="9">
@@ -6454,10 +6360,10 @@
         </is>
       </c>
       <c r="E9" s="4" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>4</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="10">
@@ -6482,10 +6388,10 @@
         </is>
       </c>
       <c r="E10" s="6" t="n">
-        <v>70</v>
+        <v>45</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>4.1</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="11">
@@ -6510,10 +6416,10 @@
         </is>
       </c>
       <c r="E11" s="4" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>4</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="12">
@@ -6538,10 +6444,10 @@
         </is>
       </c>
       <c r="E12" s="6" t="n">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="F12" s="6" t="n">
-        <v>4.12</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="13">
@@ -6566,10 +6472,10 @@
         </is>
       </c>
       <c r="E13" s="4" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>4.33</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="14">
@@ -6594,10 +6500,10 @@
         </is>
       </c>
       <c r="E14" s="6" t="n">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="F14" s="6" t="n">
-        <v>3.8</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="15">
@@ -6622,7 +6528,7 @@
         </is>
       </c>
       <c r="E15" s="4" t="n">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="F15" s="4" t="n">
         <v>4</v>
@@ -6650,10 +6556,10 @@
         </is>
       </c>
       <c r="E16" s="6" t="n">
-        <v>95</v>
+        <v>70</v>
       </c>
       <c r="F16" s="6" t="n">
-        <v>3.88</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="17">
@@ -6678,10 +6584,10 @@
         </is>
       </c>
       <c r="E17" s="4" t="n">
-        <v>75</v>
+        <v>95</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>4</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="18">
@@ -6706,10 +6612,10 @@
         </is>
       </c>
       <c r="E18" s="6" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F18" s="6" t="n">
-        <v>4.33</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="19">
@@ -6734,10 +6640,10 @@
         </is>
       </c>
       <c r="E19" s="4" t="n">
-        <v>75</v>
+        <v>60</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>4.22</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="20">
@@ -6765,7 +6671,7 @@
         <v>75</v>
       </c>
       <c r="F20" s="6" t="n">
-        <v>3.8</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="21">
@@ -6790,10 +6696,10 @@
         </is>
       </c>
       <c r="E21" s="4" t="n">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>4</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="22">
@@ -6818,10 +6724,10 @@
         </is>
       </c>
       <c r="E22" s="6" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="F22" s="6" t="n">
-        <v>4.57</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="23">
@@ -6849,7 +6755,7 @@
         <v>80</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>3.57</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="24">
@@ -6874,10 +6780,10 @@
         </is>
       </c>
       <c r="E24" s="6" t="n">
-        <v>70</v>
+        <v>95</v>
       </c>
       <c r="F24" s="6" t="n">
-        <v>4.17</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="26" ht="22" customHeight="1">
@@ -6919,10 +6825,10 @@
         <v>6</v>
       </c>
       <c r="C28" s="6" t="n">
-        <v>66.7</v>
+        <v>61.7</v>
       </c>
       <c r="D28" s="6" t="n">
-        <v>3.79</v>
+        <v>3.03</v>
       </c>
     </row>
     <row r="29">
@@ -6935,10 +6841,10 @@
         <v>3</v>
       </c>
       <c r="C29" s="4" t="n">
-        <v>53.3</v>
+        <v>46.7</v>
       </c>
       <c r="D29" s="4" t="n">
-        <v>4.15</v>
+        <v>2.87</v>
       </c>
     </row>
     <row r="30">
@@ -6951,10 +6857,10 @@
         <v>4</v>
       </c>
       <c r="C30" s="6" t="n">
-        <v>78.8</v>
+        <v>81.2</v>
       </c>
       <c r="D30" s="6" t="n">
-        <v>3.92</v>
+        <v>3.12</v>
       </c>
     </row>
     <row r="31">
@@ -6967,10 +6873,10 @@
         <v>4</v>
       </c>
       <c r="C31" s="4" t="n">
-        <v>72.5</v>
+        <v>70</v>
       </c>
       <c r="D31" s="4" t="n">
-        <v>4.09</v>
+        <v>3</v>
       </c>
     </row>
     <row r="32">
@@ -6983,10 +6889,10 @@
         <v>2</v>
       </c>
       <c r="C32" s="6" t="n">
-        <v>77.5</v>
+        <v>80</v>
       </c>
       <c r="D32" s="6" t="n">
-        <v>4.07</v>
+        <v>3.15</v>
       </c>
     </row>
     <row r="33">
@@ -6999,10 +6905,10 @@
         <v>1</v>
       </c>
       <c r="C33" s="4" t="n">
-        <v>70</v>
+        <v>95</v>
       </c>
       <c r="D33" s="4" t="n">
-        <v>4.17</v>
+        <v>3.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>